<commit_message>
data set cleaned q1-1
</commit_message>
<xml_diff>
--- a/DATA_SETS/q1-1.xlsx
+++ b/DATA_SETS/q1-1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\farha\KRMU\GitHub\SEM-2-MINOR_PROJECT\DATA_SETS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAB7D9FB-8555-4736-8038-E6DCAEAC3146}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{500E4315-AE25-47E5-949F-FA186D948AF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10886" yWindow="0" windowWidth="11143" windowHeight="13080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Books" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="233">
   <si>
     <t>Book_ID</t>
   </si>
@@ -43,9 +43,6 @@
     <t>B001</t>
   </si>
   <si>
-    <t>Book Title 1</t>
-  </si>
-  <si>
     <t>Napoleon Hill</t>
   </si>
   <si>
@@ -55,9 +52,6 @@
     <t>B002</t>
   </si>
   <si>
-    <t>Book Title 2</t>
-  </si>
-  <si>
     <t>Robert Kiyosaki</t>
   </si>
   <si>
@@ -67,9 +61,6 @@
     <t>B003</t>
   </si>
   <si>
-    <t>Book Title 3</t>
-  </si>
-  <si>
     <t>Colleen Hoover</t>
   </si>
   <si>
@@ -79,9 +70,6 @@
     <t>B004</t>
   </si>
   <si>
-    <t>Book Title 4</t>
-  </si>
-  <si>
     <t>F. Scott Fitzgerald</t>
   </si>
   <si>
@@ -91,24 +79,15 @@
     <t>B005</t>
   </si>
   <si>
-    <t>Book Title 5</t>
-  </si>
-  <si>
     <t>B006</t>
   </si>
   <si>
-    <t>Book Title 6</t>
-  </si>
-  <si>
     <t>Mark Manson</t>
   </si>
   <si>
     <t>B007</t>
   </si>
   <si>
-    <t>Book Title 7</t>
-  </si>
-  <si>
     <t>Alex Michaelides</t>
   </si>
   <si>
@@ -118,18 +97,12 @@
     <t>B008</t>
   </si>
   <si>
-    <t>Book Title 8</t>
-  </si>
-  <si>
     <t>Stephen King</t>
   </si>
   <si>
     <t>B009</t>
   </si>
   <si>
-    <t>Book Title 9</t>
-  </si>
-  <si>
     <t>Robin Sharma</t>
   </si>
   <si>
@@ -139,602 +112,632 @@
     <t>B010</t>
   </si>
   <si>
-    <t>Book Title 10</t>
-  </si>
-  <si>
     <t>B011</t>
   </si>
   <si>
-    <t>Book Title 11</t>
-  </si>
-  <si>
     <t>Fiction</t>
   </si>
   <si>
     <t>B012</t>
   </si>
   <si>
-    <t>Book Title 12</t>
-  </si>
-  <si>
     <t>Yuval Noah Harari</t>
   </si>
   <si>
     <t>B013</t>
   </si>
   <si>
-    <t>Book Title 13</t>
-  </si>
-  <si>
     <t>B014</t>
   </si>
   <si>
-    <t>Book Title 14</t>
-  </si>
-  <si>
     <t>B015</t>
   </si>
   <si>
-    <t>Book Title 15</t>
-  </si>
-  <si>
     <t>J.K. Rowling</t>
   </si>
   <si>
     <t>B016</t>
   </si>
   <si>
-    <t>Book Title 16</t>
-  </si>
-  <si>
     <t>Science Fiction</t>
   </si>
   <si>
     <t>B017</t>
   </si>
   <si>
-    <t>Book Title 17</t>
-  </si>
-  <si>
     <t>Paulo Coelho</t>
   </si>
   <si>
     <t>B018</t>
   </si>
   <si>
-    <t>Book Title 18</t>
-  </si>
-  <si>
     <t>B019</t>
   </si>
   <si>
-    <t>Book Title 19</t>
-  </si>
-  <si>
     <t>George Orwell</t>
   </si>
   <si>
     <t>B020</t>
   </si>
   <si>
-    <t>Book Title 20</t>
-  </si>
-  <si>
     <t>B021</t>
   </si>
   <si>
-    <t>Book Title 21</t>
-  </si>
-  <si>
     <t>B022</t>
   </si>
   <si>
-    <t>Book Title 22</t>
-  </si>
-  <si>
     <t>B023</t>
   </si>
   <si>
-    <t>Book Title 23</t>
-  </si>
-  <si>
     <t>History</t>
   </si>
   <si>
     <t>B024</t>
   </si>
   <si>
-    <t>Book Title 24</t>
-  </si>
-  <si>
     <t>Mystery</t>
   </si>
   <si>
     <t>B025</t>
   </si>
   <si>
-    <t>Book Title 25</t>
-  </si>
-  <si>
     <t>B026</t>
   </si>
   <si>
-    <t>Book Title 26</t>
-  </si>
-  <si>
     <t>B027</t>
   </si>
   <si>
-    <t>Book Title 27</t>
-  </si>
-  <si>
     <t>Agatha Christie</t>
   </si>
   <si>
     <t>B028</t>
   </si>
   <si>
-    <t>Book Title 28</t>
-  </si>
-  <si>
     <t>B029</t>
   </si>
   <si>
-    <t>Book Title 29</t>
-  </si>
-  <si>
     <t>B030</t>
   </si>
   <si>
-    <t>Book Title 30</t>
-  </si>
-  <si>
     <t>B031</t>
   </si>
   <si>
-    <t>Book Title 31</t>
-  </si>
-  <si>
     <t>B032</t>
   </si>
   <si>
-    <t>Book Title 32</t>
-  </si>
-  <si>
     <t>B033</t>
   </si>
   <si>
-    <t>Book Title 33</t>
-  </si>
-  <si>
     <t>B034</t>
   </si>
   <si>
-    <t>Book Title 34</t>
-  </si>
-  <si>
     <t>B035</t>
   </si>
   <si>
-    <t>Book Title 35</t>
-  </si>
-  <si>
     <t>J.R.R. Tolkien</t>
   </si>
   <si>
     <t>B036</t>
   </si>
   <si>
-    <t>Book Title 36</t>
-  </si>
-  <si>
     <t>B037</t>
   </si>
   <si>
-    <t>Book Title 37</t>
-  </si>
-  <si>
     <t>B038</t>
   </si>
   <si>
-    <t>Book Title 38</t>
-  </si>
-  <si>
     <t>B039</t>
   </si>
   <si>
-    <t>Book Title 39</t>
-  </si>
-  <si>
     <t>B040</t>
   </si>
   <si>
-    <t>Book Title 40</t>
-  </si>
-  <si>
     <t>B041</t>
   </si>
   <si>
-    <t>Book Title 41</t>
-  </si>
-  <si>
     <t>Dale Carnegie</t>
   </si>
   <si>
     <t>B042</t>
   </si>
   <si>
-    <t>Book Title 42</t>
-  </si>
-  <si>
     <t>Dan Brown</t>
   </si>
   <si>
     <t>B043</t>
   </si>
   <si>
-    <t>Book Title 43</t>
-  </si>
-  <si>
     <t>B044</t>
   </si>
   <si>
-    <t>Book Title 44</t>
-  </si>
-  <si>
     <t>B045</t>
   </si>
   <si>
-    <t>Book Title 45</t>
-  </si>
-  <si>
     <t>B046</t>
   </si>
   <si>
-    <t>Book Title 46</t>
-  </si>
-  <si>
     <t>B047</t>
   </si>
   <si>
-    <t>Book Title 47</t>
-  </si>
-  <si>
     <t>B048</t>
   </si>
   <si>
-    <t>Book Title 48</t>
-  </si>
-  <si>
     <t>B049</t>
   </si>
   <si>
-    <t>Book Title 49</t>
-  </si>
-  <si>
     <t>B050</t>
   </si>
   <si>
-    <t>Book Title 50</t>
-  </si>
-  <si>
     <t>B051</t>
   </si>
   <si>
-    <t>Book Title 51</t>
-  </si>
-  <si>
     <t>B052</t>
   </si>
   <si>
-    <t>Book Title 52</t>
-  </si>
-  <si>
     <t>B053</t>
   </si>
   <si>
-    <t>Book Title 53</t>
-  </si>
-  <si>
     <t>B054</t>
   </si>
   <si>
-    <t>Book Title 54</t>
-  </si>
-  <si>
     <t>B055</t>
   </si>
   <si>
-    <t>Book Title 55</t>
-  </si>
-  <si>
     <t>James Clear</t>
   </si>
   <si>
     <t>B056</t>
   </si>
   <si>
-    <t>Book Title 56</t>
-  </si>
-  <si>
     <t>B057</t>
   </si>
   <si>
-    <t>Book Title 57</t>
-  </si>
-  <si>
     <t>B058</t>
   </si>
   <si>
-    <t>Book Title 58</t>
-  </si>
-  <si>
     <t>B059</t>
   </si>
   <si>
-    <t>Book Title 59</t>
-  </si>
-  <si>
     <t>B060</t>
   </si>
   <si>
-    <t>Book Title 60</t>
-  </si>
-  <si>
     <t>B061</t>
   </si>
   <si>
-    <t>Book Title 61</t>
-  </si>
-  <si>
     <t>B062</t>
   </si>
   <si>
-    <t>Book Title 62</t>
-  </si>
-  <si>
     <t>B063</t>
   </si>
   <si>
-    <t>Book Title 63</t>
-  </si>
-  <si>
     <t>B064</t>
   </si>
   <si>
-    <t>Book Title 64</t>
-  </si>
-  <si>
     <t>B065</t>
   </si>
   <si>
-    <t>Book Title 65</t>
-  </si>
-  <si>
     <t>B066</t>
   </si>
   <si>
-    <t>Book Title 66</t>
-  </si>
-  <si>
     <t>B067</t>
   </si>
   <si>
-    <t>Book Title 67</t>
-  </si>
-  <si>
     <t>B068</t>
   </si>
   <si>
-    <t>Book Title 68</t>
-  </si>
-  <si>
     <t>B069</t>
   </si>
   <si>
-    <t>Book Title 69</t>
-  </si>
-  <si>
     <t>B070</t>
   </si>
   <si>
-    <t>Book Title 70</t>
-  </si>
-  <si>
     <t>B071</t>
   </si>
   <si>
-    <t>Book Title 71</t>
-  </si>
-  <si>
     <t>B072</t>
   </si>
   <si>
-    <t>Book Title 72</t>
-  </si>
-  <si>
     <t>B073</t>
   </si>
   <si>
-    <t>Book Title 73</t>
-  </si>
-  <si>
     <t>B074</t>
   </si>
   <si>
-    <t>Book Title 74</t>
-  </si>
-  <si>
     <t>B075</t>
   </si>
   <si>
-    <t>Book Title 75</t>
-  </si>
-  <si>
     <t>B076</t>
   </si>
   <si>
-    <t>Book Title 76</t>
-  </si>
-  <si>
     <t>B077</t>
   </si>
   <si>
-    <t>Book Title 77</t>
-  </si>
-  <si>
     <t>B078</t>
   </si>
   <si>
-    <t>Book Title 78</t>
-  </si>
-  <si>
     <t>B079</t>
   </si>
   <si>
-    <t>Book Title 79</t>
-  </si>
-  <si>
     <t>B080</t>
   </si>
   <si>
-    <t>Book Title 80</t>
-  </si>
-  <si>
     <t>B081</t>
   </si>
   <si>
-    <t>Book Title 81</t>
-  </si>
-  <si>
     <t>B082</t>
   </si>
   <si>
-    <t>Book Title 82</t>
-  </si>
-  <si>
     <t>B083</t>
   </si>
   <si>
-    <t>Book Title 83</t>
-  </si>
-  <si>
     <t>B084</t>
   </si>
   <si>
-    <t>Book Title 84</t>
-  </si>
-  <si>
     <t>B085</t>
   </si>
   <si>
-    <t>Book Title 85</t>
-  </si>
-  <si>
     <t>B086</t>
   </si>
   <si>
-    <t>Book Title 86</t>
-  </si>
-  <si>
     <t>B087</t>
   </si>
   <si>
-    <t>Book Title 87</t>
-  </si>
-  <si>
     <t>B088</t>
   </si>
   <si>
-    <t>Book Title 88</t>
-  </si>
-  <si>
     <t>Harper Lee</t>
   </si>
   <si>
     <t>B089</t>
   </si>
   <si>
-    <t>Book Title 89</t>
-  </si>
-  <si>
     <t>B090</t>
   </si>
   <si>
-    <t>Book Title 90</t>
-  </si>
-  <si>
     <t>B091</t>
   </si>
   <si>
-    <t>Book Title 91</t>
-  </si>
-  <si>
     <t>B092</t>
   </si>
   <si>
-    <t>Book Title 92</t>
-  </si>
-  <si>
     <t>B093</t>
   </si>
   <si>
-    <t>Book Title 93</t>
-  </si>
-  <si>
     <t>B094</t>
   </si>
   <si>
-    <t>Book Title 94</t>
-  </si>
-  <si>
     <t>B095</t>
   </si>
   <si>
-    <t>Book Title 95</t>
-  </si>
-  <si>
     <t>B096</t>
   </si>
   <si>
-    <t>Book Title 96</t>
-  </si>
-  <si>
     <t>B097</t>
   </si>
   <si>
-    <t>Book Title 97</t>
-  </si>
-  <si>
     <t>B098</t>
   </si>
   <si>
-    <t>Book Title 98</t>
-  </si>
-  <si>
     <t>B099</t>
   </si>
   <si>
-    <t>Book Title 99</t>
-  </si>
-  <si>
     <t>B100</t>
   </si>
   <si>
-    <t>Book Title 100</t>
+    <t>Don Quixote</t>
+  </si>
+  <si>
+    <t>To Kill a Mockingbird</t>
+  </si>
+  <si>
+    <t>Pride and Prejudice</t>
+  </si>
+  <si>
+    <t>The Great Gatsby</t>
+  </si>
+  <si>
+    <t>The Catcher in the Rye</t>
+  </si>
+  <si>
+    <t>The Lord of the Rings</t>
+  </si>
+  <si>
+    <t>The Hobbit</t>
+  </si>
+  <si>
+    <t>Jane Eyre</t>
+  </si>
+  <si>
+    <t>Wuthering Heights</t>
+  </si>
+  <si>
+    <t>Animal Farm</t>
+  </si>
+  <si>
+    <t>Fahrenheit 451</t>
+  </si>
+  <si>
+    <t>The Grapes of Wrath</t>
+  </si>
+  <si>
+    <t>Brave New World</t>
+  </si>
+  <si>
+    <t>The Book Thief</t>
+  </si>
+  <si>
+    <t>The Kite Runner</t>
+  </si>
+  <si>
+    <t>Moby Dick</t>
+  </si>
+  <si>
+    <t>War and Peace</t>
+  </si>
+  <si>
+    <t>Anna Karenina</t>
+  </si>
+  <si>
+    <t>The Odyssey</t>
+  </si>
+  <si>
+    <t>The Iliad</t>
+  </si>
+  <si>
+    <t>Crime and Punishment</t>
+  </si>
+  <si>
+    <t>The Brothers Karamazov</t>
+  </si>
+  <si>
+    <t>One Hundred Years of Solitude</t>
+  </si>
+  <si>
+    <t>Ulysses</t>
+  </si>
+  <si>
+    <t>The Picture of Dorian Gray</t>
+  </si>
+  <si>
+    <t>Dracula</t>
+  </si>
+  <si>
+    <t>Frankenstein</t>
+  </si>
+  <si>
+    <t>The Adventures of Huckleberry Finn</t>
+  </si>
+  <si>
+    <t>Alice's Adventures in Wonderland</t>
+  </si>
+  <si>
+    <t>Les Misérables</t>
+  </si>
+  <si>
+    <t>The Count of Monte Cristo</t>
+  </si>
+  <si>
+    <t>The Three Musketeers</t>
+  </si>
+  <si>
+    <t>The Stranger</t>
+  </si>
+  <si>
+    <t>The Trial</t>
+  </si>
+  <si>
+    <t>The Metamorphosis</t>
+  </si>
+  <si>
+    <t>The Old Man and the Sea</t>
+  </si>
+  <si>
+    <t>A Farewell to Arms</t>
+  </si>
+  <si>
+    <t>For Whom the Bell Tolls</t>
+  </si>
+  <si>
+    <t>Gone with the Wind</t>
+  </si>
+  <si>
+    <t>Great Expectations</t>
+  </si>
+  <si>
+    <t>A Tale of Two Cities</t>
+  </si>
+  <si>
+    <t>Oliver Twist</t>
+  </si>
+  <si>
+    <t>David Copperfield</t>
+  </si>
+  <si>
+    <t>Little Women</t>
+  </si>
+  <si>
+    <t>The Secret Garden</t>
+  </si>
+  <si>
+    <t>The Chronicles of Narnia</t>
+  </si>
+  <si>
+    <t>The Lion, the Witch and the Wardrobe</t>
+  </si>
+  <si>
+    <t>The Alchemist</t>
+  </si>
+  <si>
+    <t>The Handmaid's Tale</t>
+  </si>
+  <si>
+    <t>The Road</t>
+  </si>
+  <si>
+    <t>Blood Meridian</t>
+  </si>
+  <si>
+    <t>Beloved</t>
+  </si>
+  <si>
+    <t>Sula</t>
+  </si>
+  <si>
+    <t>The Color Purple</t>
+  </si>
+  <si>
+    <t>Invisible Man</t>
+  </si>
+  <si>
+    <t>Catch-22</t>
+  </si>
+  <si>
+    <t>Slaughterhouse-Five</t>
+  </si>
+  <si>
+    <t>The Bell Jar</t>
+  </si>
+  <si>
+    <t>Lolita</t>
+  </si>
+  <si>
+    <t>Siddhartha</t>
+  </si>
+  <si>
+    <t>The Catch in the Rye</t>
+  </si>
+  <si>
+    <t>Of Mice and Men</t>
+  </si>
+  <si>
+    <t>The Sun Also Rises</t>
+  </si>
+  <si>
+    <t>Things Fall Apart</t>
+  </si>
+  <si>
+    <t>Midnight's Children</t>
+  </si>
+  <si>
+    <t>The God of Small Things</t>
+  </si>
+  <si>
+    <t>Life of Pi</t>
+  </si>
+  <si>
+    <t>The Shadow of the Wind</t>
+  </si>
+  <si>
+    <t>Memoirs of a Geisha</t>
+  </si>
+  <si>
+    <t>The Girl with the Dragon Tattoo</t>
+  </si>
+  <si>
+    <t>The Da Vinci Code</t>
+  </si>
+  <si>
+    <t>The Hunger Games</t>
+  </si>
+  <si>
+    <t>Divergent</t>
+  </si>
+  <si>
+    <t>The Fault in Our Stars</t>
+  </si>
+  <si>
+    <t>Harry Potter and the Sorcerer's Stone</t>
+  </si>
+  <si>
+    <t>The Poisonwood Bible</t>
+  </si>
+  <si>
+    <t>The Help</t>
+  </si>
+  <si>
+    <t>The Goldfinch</t>
+  </si>
+  <si>
+    <t>A Little Life</t>
+  </si>
+  <si>
+    <t>Educated</t>
+  </si>
+  <si>
+    <t>Becoming</t>
+  </si>
+  <si>
+    <t>Sapiens: A Brief History of Humankind</t>
+  </si>
+  <si>
+    <t>Thinking, Fast and Slow</t>
+  </si>
+  <si>
+    <t>The 7 Habits of Highly Effective People</t>
+  </si>
+  <si>
+    <t>How to Win Friends and Influence People</t>
+  </si>
+  <si>
+    <t>The Power of Habit</t>
+  </si>
+  <si>
+    <t>Man's Search for Meaning</t>
+  </si>
+  <si>
+    <t>The Diary of a Young Girl</t>
+  </si>
+  <si>
+    <t>Night</t>
+  </si>
+  <si>
+    <t>The Glass Castle</t>
+  </si>
+  <si>
+    <t>Wild</t>
+  </si>
+  <si>
+    <t>Into the Wild</t>
+  </si>
+  <si>
+    <t>The Immortal Life of Henrietta Lacks</t>
+  </si>
+  <si>
+    <t>The Emperor of All Maladies</t>
+  </si>
+  <si>
+    <t>Quiet: The Power of Introverts</t>
+  </si>
+  <si>
+    <t>Guns, Germs, and Steel</t>
+  </si>
+  <si>
+    <t>A Brief History of Time</t>
+  </si>
+  <si>
+    <t>The Selfish Gene</t>
+  </si>
+  <si>
+    <t>Meditations</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -757,8 +760,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1095,14 +1104,14 @@
       <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
       </c>
       <c r="E2">
         <v>133</v>
@@ -1111,18 +1120,18 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
         <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
       </c>
       <c r="E3">
         <v>147</v>
@@ -1133,16 +1142,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2">
+        <v>1984</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
         <v>14</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" t="s">
-        <v>17</v>
       </c>
       <c r="E4">
         <v>133</v>
@@ -1151,18 +1160,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" t="s">
-        <v>19</v>
+        <v>15</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>136</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E5">
         <v>85</v>
@@ -1173,16 +1182,16 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" t="s">
-        <v>23</v>
+        <v>18</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>137</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E6">
         <v>58</v>
@@ -1191,18 +1200,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" t="s">
-        <v>25</v>
+        <v>19</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>138</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E7">
         <v>122</v>
@@ -1211,18 +1220,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" t="s">
-        <v>28</v>
+        <v>21</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>139</v>
       </c>
       <c r="C8" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D8" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E8">
         <v>117</v>
@@ -1233,16 +1242,16 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" t="s">
-        <v>32</v>
+        <v>24</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>140</v>
       </c>
       <c r="C9" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D9" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E9">
         <v>53</v>
@@ -1253,16 +1262,16 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
-        <v>34</v>
-      </c>
-      <c r="B10" t="s">
-        <v>35</v>
+        <v>26</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>141</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="D10" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="E10">
         <v>137</v>
@@ -1273,16 +1282,16 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" t="s">
-        <v>39</v>
+        <v>29</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>142</v>
       </c>
       <c r="C11" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E11">
         <v>130</v>
@@ -1293,16 +1302,16 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
-        <v>40</v>
-      </c>
-      <c r="B12" t="s">
-        <v>41</v>
+        <v>30</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>143</v>
       </c>
       <c r="C12" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D12" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="E12">
         <v>54</v>
@@ -1313,16 +1322,16 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
-        <v>43</v>
-      </c>
-      <c r="B13" t="s">
-        <v>44</v>
+        <v>32</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>144</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="D13" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E13">
         <v>126</v>
@@ -1331,18 +1340,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
-        <v>46</v>
-      </c>
-      <c r="B14" t="s">
-        <v>47</v>
+        <v>34</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>145</v>
       </c>
       <c r="C14" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D14" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E14">
         <v>137</v>
@@ -1353,16 +1362,16 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B15" t="s">
-        <v>49</v>
+        <v>35</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>146</v>
       </c>
       <c r="C15" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D15" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E15">
         <v>123</v>
@@ -1373,16 +1382,16 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
-        <v>50</v>
-      </c>
-      <c r="B16" t="s">
-        <v>51</v>
+        <v>36</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>147</v>
       </c>
       <c r="C16" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="D16" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E16">
         <v>116</v>
@@ -1393,16 +1402,16 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
-        <v>53</v>
-      </c>
-      <c r="B17" t="s">
-        <v>54</v>
+        <v>38</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>148</v>
       </c>
       <c r="C17" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="D17" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="E17">
         <v>69</v>
@@ -1413,16 +1422,16 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
-        <v>56</v>
-      </c>
-      <c r="B18" t="s">
-        <v>57</v>
+        <v>40</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>149</v>
       </c>
       <c r="C18" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="D18" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="E18">
         <v>92</v>
@@ -1433,16 +1442,16 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
-        <v>59</v>
-      </c>
-      <c r="B19" t="s">
-        <v>60</v>
+        <v>42</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>150</v>
       </c>
       <c r="C19" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D19" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E19">
         <v>111</v>
@@ -1453,16 +1462,16 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
-        <v>61</v>
-      </c>
-      <c r="B20" t="s">
-        <v>62</v>
+        <v>43</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>151</v>
       </c>
       <c r="C20" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="D20" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E20">
         <v>87</v>
@@ -1473,16 +1482,16 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
-        <v>64</v>
-      </c>
-      <c r="B21" t="s">
-        <v>65</v>
+        <v>45</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>152</v>
       </c>
       <c r="C21" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="D21" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="E21">
         <v>138</v>
@@ -1493,16 +1502,16 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
-        <v>66</v>
-      </c>
-      <c r="B22" t="s">
-        <v>67</v>
+        <v>46</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>153</v>
       </c>
       <c r="C22" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D22" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="E22">
         <v>141</v>
@@ -1511,18 +1520,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
-        <v>68</v>
-      </c>
-      <c r="B23" t="s">
-        <v>69</v>
+        <v>47</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>154</v>
       </c>
       <c r="C23" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D23" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="E23">
         <v>108</v>
@@ -1531,18 +1540,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
-        <v>70</v>
-      </c>
-      <c r="B24" t="s">
-        <v>71</v>
+        <v>48</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>155</v>
       </c>
       <c r="C24" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="D24" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="E24">
         <v>136</v>
@@ -1551,18 +1560,18 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
-        <v>73</v>
-      </c>
-      <c r="B25" t="s">
-        <v>74</v>
+        <v>50</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>156</v>
       </c>
       <c r="C25" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="D25" t="s">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="E25">
         <v>124</v>
@@ -1573,16 +1582,16 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
-        <v>76</v>
-      </c>
-      <c r="B26" t="s">
-        <v>77</v>
+        <v>52</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>157</v>
       </c>
       <c r="C26" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D26" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="E26">
         <v>53</v>
@@ -1591,18 +1600,18 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
-        <v>78</v>
-      </c>
-      <c r="B27" t="s">
-        <v>79</v>
+        <v>53</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>158</v>
       </c>
       <c r="C27" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D27" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E27">
         <v>84</v>
@@ -1613,16 +1622,16 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
-        <v>80</v>
-      </c>
-      <c r="B28" t="s">
-        <v>81</v>
+        <v>54</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>159</v>
       </c>
       <c r="C28" t="s">
-        <v>82</v>
+        <v>55</v>
       </c>
       <c r="D28" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E28">
         <v>63</v>
@@ -1633,16 +1642,16 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
-        <v>83</v>
-      </c>
-      <c r="B29" t="s">
-        <v>84</v>
+        <v>56</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>160</v>
       </c>
       <c r="C29" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="D29" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E29">
         <v>124</v>
@@ -1651,18 +1660,18 @@
         <v>7</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
-        <v>85</v>
-      </c>
-      <c r="B30" t="s">
-        <v>86</v>
+        <v>57</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>161</v>
       </c>
       <c r="C30" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D30" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="E30">
         <v>62</v>
@@ -1671,18 +1680,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
-        <v>87</v>
-      </c>
-      <c r="B31" t="s">
-        <v>88</v>
+        <v>58</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>162</v>
       </c>
       <c r="C31" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="D31" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="E31">
         <v>132</v>
@@ -1693,16 +1702,16 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
-        <v>89</v>
-      </c>
-      <c r="B32" t="s">
-        <v>90</v>
+        <v>59</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>163</v>
       </c>
       <c r="C32" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D32" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E32">
         <v>150</v>
@@ -1711,18 +1720,18 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
-        <v>91</v>
-      </c>
-      <c r="B33" t="s">
-        <v>92</v>
+        <v>60</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>164</v>
       </c>
       <c r="C33" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D33" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E33">
         <v>148</v>
@@ -1731,18 +1740,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
-        <v>93</v>
-      </c>
-      <c r="B34" t="s">
-        <v>94</v>
+        <v>61</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>165</v>
       </c>
       <c r="C34" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D34" t="s">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="E34">
         <v>126</v>
@@ -1753,16 +1762,16 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
-        <v>95</v>
-      </c>
-      <c r="B35" t="s">
-        <v>96</v>
+        <v>62</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>166</v>
       </c>
       <c r="C35" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="D35" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="E35">
         <v>80</v>
@@ -1773,16 +1782,16 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
-        <v>97</v>
-      </c>
-      <c r="B36" t="s">
-        <v>98</v>
+        <v>63</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>167</v>
       </c>
       <c r="C36" t="s">
-        <v>99</v>
+        <v>64</v>
       </c>
       <c r="D36" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="E36">
         <v>61</v>
@@ -1791,18 +1800,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
-        <v>100</v>
-      </c>
-      <c r="B37" t="s">
-        <v>101</v>
+        <v>65</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>168</v>
       </c>
       <c r="C37" t="s">
-        <v>82</v>
+        <v>55</v>
       </c>
       <c r="D37" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E37">
         <v>58</v>
@@ -1811,18 +1820,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
-        <v>102</v>
-      </c>
-      <c r="B38" t="s">
-        <v>103</v>
+        <v>66</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>169</v>
       </c>
       <c r="C38" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="D38" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E38">
         <v>78</v>
@@ -1831,18 +1840,18 @@
         <v>7</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
-        <v>104</v>
-      </c>
-      <c r="B39" t="s">
-        <v>105</v>
+        <v>67</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>170</v>
       </c>
       <c r="C39" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D39" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E39">
         <v>96</v>
@@ -1851,18 +1860,18 @@
         <v>2</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
-        <v>106</v>
-      </c>
-      <c r="B40" t="s">
-        <v>107</v>
+        <v>68</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>171</v>
       </c>
       <c r="C40" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D40" t="s">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="E40">
         <v>91</v>
@@ -1871,18 +1880,18 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
-        <v>108</v>
-      </c>
-      <c r="B41" t="s">
-        <v>109</v>
+        <v>69</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>172</v>
       </c>
       <c r="C41" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D41" t="s">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="E41">
         <v>78</v>
@@ -1891,18 +1900,18 @@
         <v>8</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
-        <v>110</v>
-      </c>
-      <c r="B42" t="s">
-        <v>111</v>
+        <v>70</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>173</v>
       </c>
       <c r="C42" t="s">
-        <v>112</v>
+        <v>71</v>
       </c>
       <c r="D42" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E42">
         <v>145</v>
@@ -1911,18 +1920,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
-        <v>113</v>
-      </c>
-      <c r="B43" t="s">
-        <v>114</v>
+        <v>72</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>174</v>
       </c>
       <c r="C43" t="s">
-        <v>115</v>
+        <v>73</v>
       </c>
       <c r="D43" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="E43">
         <v>74</v>
@@ -1933,16 +1942,16 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
-        <v>116</v>
-      </c>
-      <c r="B44" t="s">
-        <v>117</v>
+        <v>74</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>175</v>
       </c>
       <c r="C44" t="s">
-        <v>115</v>
+        <v>73</v>
       </c>
       <c r="D44" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E44">
         <v>97</v>
@@ -1953,16 +1962,16 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
-        <v>118</v>
-      </c>
-      <c r="B45" t="s">
-        <v>119</v>
+        <v>75</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>176</v>
       </c>
       <c r="C45" t="s">
-        <v>115</v>
+        <v>73</v>
       </c>
       <c r="D45" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E45">
         <v>118</v>
@@ -1973,16 +1982,16 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
-        <v>120</v>
-      </c>
-      <c r="B46" t="s">
-        <v>121</v>
+        <v>76</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>177</v>
       </c>
       <c r="C46" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D46" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="E46">
         <v>103</v>
@@ -1991,18 +2000,18 @@
         <v>3</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
-        <v>122</v>
-      </c>
-      <c r="B47" t="s">
-        <v>123</v>
+        <v>77</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>178</v>
       </c>
       <c r="C47" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D47" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E47">
         <v>116</v>
@@ -2011,18 +2020,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A48" t="s">
-        <v>124</v>
-      </c>
-      <c r="B48" t="s">
-        <v>125</v>
+        <v>78</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>179</v>
       </c>
       <c r="C48" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="D48" t="s">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="E48">
         <v>122</v>
@@ -2031,18 +2040,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:6" ht="38.15" x14ac:dyDescent="0.4">
       <c r="A49" t="s">
-        <v>126</v>
-      </c>
-      <c r="B49" t="s">
-        <v>127</v>
+        <v>79</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>180</v>
       </c>
       <c r="C49" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D49" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="E49">
         <v>60</v>
@@ -2053,16 +2062,16 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A50" t="s">
-        <v>128</v>
-      </c>
-      <c r="B50" t="s">
-        <v>129</v>
+        <v>80</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>181</v>
       </c>
       <c r="C50" t="s">
-        <v>115</v>
+        <v>73</v>
       </c>
       <c r="D50" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="E50">
         <v>94</v>
@@ -2071,18 +2080,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
-        <v>130</v>
-      </c>
-      <c r="B51" t="s">
-        <v>131</v>
+        <v>81</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>182</v>
       </c>
       <c r="C51" t="s">
-        <v>115</v>
+        <v>73</v>
       </c>
       <c r="D51" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E51">
         <v>64</v>
@@ -2093,16 +2102,16 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
-        <v>132</v>
-      </c>
-      <c r="B52" t="s">
-        <v>133</v>
+        <v>82</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>183</v>
       </c>
       <c r="C52" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D52" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="E52">
         <v>126</v>
@@ -2113,16 +2122,16 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
-        <v>134</v>
-      </c>
-      <c r="B53" t="s">
-        <v>135</v>
+        <v>83</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>184</v>
       </c>
       <c r="C53" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D53" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="E53">
         <v>51</v>
@@ -2133,16 +2142,16 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
-        <v>136</v>
-      </c>
-      <c r="B54" t="s">
-        <v>137</v>
+        <v>84</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>185</v>
       </c>
       <c r="C54" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D54" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E54">
         <v>112</v>
@@ -2153,16 +2162,16 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
-        <v>138</v>
-      </c>
-      <c r="B55" t="s">
-        <v>139</v>
+        <v>85</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>186</v>
       </c>
       <c r="C55" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D55" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="E55">
         <v>98</v>
@@ -2173,16 +2182,16 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
-        <v>140</v>
-      </c>
-      <c r="B56" t="s">
-        <v>141</v>
+        <v>86</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>187</v>
       </c>
       <c r="C56" t="s">
-        <v>142</v>
+        <v>87</v>
       </c>
       <c r="D56" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E56">
         <v>60</v>
@@ -2193,16 +2202,16 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
-        <v>143</v>
-      </c>
-      <c r="B57" t="s">
-        <v>144</v>
+        <v>88</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>188</v>
       </c>
       <c r="C57" t="s">
-        <v>112</v>
+        <v>71</v>
       </c>
       <c r="D57" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E57">
         <v>76</v>
@@ -2213,16 +2222,16 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A58" t="s">
-        <v>145</v>
-      </c>
-      <c r="B58" t="s">
-        <v>146</v>
+        <v>89</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>189</v>
       </c>
       <c r="C58" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D58" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="E58">
         <v>126</v>
@@ -2231,18 +2240,18 @@
         <v>3</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A59" t="s">
-        <v>147</v>
-      </c>
-      <c r="B59" t="s">
-        <v>148</v>
+        <v>90</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>190</v>
       </c>
       <c r="C59" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D59" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E59">
         <v>148</v>
@@ -2253,16 +2262,16 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A60" t="s">
-        <v>149</v>
-      </c>
-      <c r="B60" t="s">
-        <v>150</v>
+        <v>91</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>191</v>
       </c>
       <c r="C60" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D60" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E60">
         <v>77</v>
@@ -2273,16 +2282,16 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A61" t="s">
-        <v>151</v>
-      </c>
-      <c r="B61" t="s">
-        <v>152</v>
+        <v>92</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>192</v>
       </c>
       <c r="C61" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D61" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E61">
         <v>82</v>
@@ -2293,16 +2302,16 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A62" t="s">
-        <v>153</v>
-      </c>
-      <c r="B62" t="s">
-        <v>154</v>
+        <v>93</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>193</v>
       </c>
       <c r="C62" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="D62" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E62">
         <v>144</v>
@@ -2311,18 +2320,18 @@
         <v>4</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A63" t="s">
-        <v>155</v>
-      </c>
-      <c r="B63" t="s">
-        <v>156</v>
+        <v>94</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>194</v>
       </c>
       <c r="C63" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="D63" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="E63">
         <v>141</v>
@@ -2333,16 +2342,16 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A64" t="s">
-        <v>157</v>
-      </c>
-      <c r="B64" t="s">
-        <v>158</v>
+        <v>95</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>195</v>
       </c>
       <c r="C64" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="D64" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="E64">
         <v>108</v>
@@ -2351,18 +2360,18 @@
         <v>7</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A65" t="s">
-        <v>159</v>
-      </c>
-      <c r="B65" t="s">
-        <v>160</v>
+        <v>96</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>196</v>
       </c>
       <c r="C65" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="D65" t="s">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="E65">
         <v>50</v>
@@ -2373,16 +2382,16 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A66" t="s">
-        <v>161</v>
-      </c>
-      <c r="B66" t="s">
-        <v>162</v>
+        <v>97</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>197</v>
       </c>
       <c r="C66" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D66" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="E66">
         <v>99</v>
@@ -2391,18 +2400,18 @@
         <v>7</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A67" t="s">
-        <v>163</v>
-      </c>
-      <c r="B67" t="s">
-        <v>164</v>
+        <v>98</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>198</v>
       </c>
       <c r="C67" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D67" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E67">
         <v>106</v>
@@ -2411,18 +2420,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A68" t="s">
-        <v>165</v>
-      </c>
-      <c r="B68" t="s">
-        <v>166</v>
+        <v>99</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>199</v>
       </c>
       <c r="C68" t="s">
-        <v>99</v>
+        <v>64</v>
       </c>
       <c r="D68" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E68">
         <v>62</v>
@@ -2433,16 +2442,16 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A69" t="s">
-        <v>167</v>
-      </c>
-      <c r="B69" t="s">
-        <v>168</v>
+        <v>100</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>200</v>
       </c>
       <c r="C69" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D69" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E69">
         <v>55</v>
@@ -2451,18 +2460,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A70" t="s">
-        <v>169</v>
-      </c>
-      <c r="B70" t="s">
-        <v>170</v>
+        <v>101</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>201</v>
       </c>
       <c r="C70" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D70" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E70">
         <v>84</v>
@@ -2471,18 +2480,18 @@
         <v>2</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A71" t="s">
-        <v>171</v>
-      </c>
-      <c r="B71" t="s">
-        <v>172</v>
+        <v>102</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>202</v>
       </c>
       <c r="C71" t="s">
-        <v>99</v>
+        <v>64</v>
       </c>
       <c r="D71" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E71">
         <v>60</v>
@@ -2491,18 +2500,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A72" t="s">
-        <v>173</v>
-      </c>
-      <c r="B72" t="s">
-        <v>174</v>
+        <v>103</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>203</v>
       </c>
       <c r="C72" t="s">
-        <v>115</v>
+        <v>73</v>
       </c>
       <c r="D72" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="E72">
         <v>51</v>
@@ -2511,18 +2520,18 @@
         <v>8</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A73" t="s">
-        <v>175</v>
-      </c>
-      <c r="B73" t="s">
-        <v>176</v>
+        <v>104</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>204</v>
       </c>
       <c r="C73" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="D73" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="E73">
         <v>69</v>
@@ -2531,18 +2540,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A74" t="s">
-        <v>177</v>
-      </c>
-      <c r="B74" t="s">
-        <v>178</v>
+        <v>105</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>205</v>
       </c>
       <c r="C74" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="D74" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E74">
         <v>135</v>
@@ -2553,16 +2562,16 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A75" t="s">
-        <v>179</v>
-      </c>
-      <c r="B75" t="s">
-        <v>180</v>
+        <v>106</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>206</v>
       </c>
       <c r="C75" t="s">
-        <v>99</v>
+        <v>64</v>
       </c>
       <c r="D75" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E75">
         <v>148</v>
@@ -2571,18 +2580,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A76" t="s">
-        <v>181</v>
-      </c>
-      <c r="B76" t="s">
-        <v>182</v>
+        <v>107</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>207</v>
       </c>
       <c r="C76" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D76" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="E76">
         <v>86</v>
@@ -2591,18 +2600,18 @@
         <v>4</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:6" ht="38.15" x14ac:dyDescent="0.4">
       <c r="A77" t="s">
-        <v>183</v>
-      </c>
-      <c r="B77" t="s">
-        <v>184</v>
+        <v>108</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>208</v>
       </c>
       <c r="C77" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="D77" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="E77">
         <v>136</v>
@@ -2611,18 +2620,18 @@
         <v>3</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A78" t="s">
-        <v>185</v>
-      </c>
-      <c r="B78" t="s">
-        <v>186</v>
+        <v>109</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>209</v>
       </c>
       <c r="C78" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D78" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E78">
         <v>71</v>
@@ -2633,16 +2642,16 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A79" t="s">
-        <v>187</v>
-      </c>
-      <c r="B79" t="s">
-        <v>188</v>
+        <v>110</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>210</v>
       </c>
       <c r="C79" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="D79" t="s">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="E79">
         <v>65</v>
@@ -2653,16 +2662,16 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A80" t="s">
-        <v>189</v>
-      </c>
-      <c r="B80" t="s">
-        <v>190</v>
+        <v>111</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>211</v>
       </c>
       <c r="C80" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="D80" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="E80">
         <v>118</v>
@@ -2673,16 +2682,16 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A81" t="s">
-        <v>191</v>
-      </c>
-      <c r="B81" t="s">
-        <v>192</v>
+        <v>112</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>212</v>
       </c>
       <c r="C81" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="D81" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="E81">
         <v>94</v>
@@ -2693,16 +2702,16 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A82" t="s">
-        <v>193</v>
-      </c>
-      <c r="B82" t="s">
-        <v>194</v>
+        <v>113</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>213</v>
       </c>
       <c r="C82" t="s">
-        <v>142</v>
+        <v>87</v>
       </c>
       <c r="D82" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="E82">
         <v>98</v>
@@ -2713,16 +2722,16 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A83" t="s">
-        <v>195</v>
-      </c>
-      <c r="B83" t="s">
-        <v>196</v>
+        <v>114</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>214</v>
       </c>
       <c r="C83" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D83" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="E83">
         <v>80</v>
@@ -2731,18 +2740,18 @@
         <v>2</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:6" ht="38.15" x14ac:dyDescent="0.4">
       <c r="A84" t="s">
-        <v>197</v>
-      </c>
-      <c r="B84" t="s">
-        <v>198</v>
+        <v>115</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>215</v>
       </c>
       <c r="C84" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D84" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E84">
         <v>145</v>
@@ -2751,18 +2760,18 @@
         <v>4</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A85" t="s">
-        <v>199</v>
-      </c>
-      <c r="B85" t="s">
-        <v>200</v>
+        <v>116</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>216</v>
       </c>
       <c r="C85" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="D85" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E85">
         <v>97</v>
@@ -2771,18 +2780,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:6" ht="38.15" x14ac:dyDescent="0.4">
       <c r="A86" t="s">
-        <v>201</v>
-      </c>
-      <c r="B86" t="s">
-        <v>202</v>
+        <v>117</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>217</v>
       </c>
       <c r="C86" t="s">
-        <v>99</v>
+        <v>64</v>
       </c>
       <c r="D86" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="E86">
         <v>137</v>
@@ -2791,18 +2800,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:6" ht="38.15" x14ac:dyDescent="0.4">
       <c r="A87" t="s">
-        <v>203</v>
-      </c>
-      <c r="B87" t="s">
-        <v>204</v>
+        <v>118</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>218</v>
       </c>
       <c r="C87" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D87" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="E87">
         <v>55</v>
@@ -2811,18 +2820,18 @@
         <v>3</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A88" t="s">
-        <v>205</v>
-      </c>
-      <c r="B88" t="s">
-        <v>206</v>
+        <v>119</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>219</v>
       </c>
       <c r="C88" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D88" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E88">
         <v>91</v>
@@ -2831,18 +2840,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A89" t="s">
-        <v>207</v>
-      </c>
-      <c r="B89" t="s">
-        <v>208</v>
+        <v>120</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>220</v>
       </c>
       <c r="C89" t="s">
-        <v>209</v>
+        <v>121</v>
       </c>
       <c r="D89" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E89">
         <v>84</v>
@@ -2851,18 +2860,18 @@
         <v>7</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A90" t="s">
-        <v>210</v>
-      </c>
-      <c r="B90" t="s">
-        <v>211</v>
+        <v>122</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>221</v>
       </c>
       <c r="C90" t="s">
-        <v>115</v>
+        <v>73</v>
       </c>
       <c r="D90" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E90">
         <v>77</v>
@@ -2873,16 +2882,16 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A91" t="s">
-        <v>212</v>
-      </c>
-      <c r="B91" t="s">
-        <v>213</v>
+        <v>123</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>222</v>
       </c>
       <c r="C91" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="D91" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E91">
         <v>103</v>
@@ -2893,16 +2902,16 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A92" t="s">
-        <v>214</v>
-      </c>
-      <c r="B92" t="s">
-        <v>215</v>
+        <v>124</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>223</v>
       </c>
       <c r="C92" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D92" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="E92">
         <v>94</v>
@@ -2913,16 +2922,16 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A93" t="s">
-        <v>216</v>
-      </c>
-      <c r="B93" t="s">
-        <v>217</v>
+        <v>125</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>224</v>
       </c>
       <c r="C93" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="D93" t="s">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="E93">
         <v>117</v>
@@ -2933,16 +2942,16 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A94" t="s">
-        <v>218</v>
-      </c>
-      <c r="B94" t="s">
-        <v>219</v>
+        <v>126</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>225</v>
       </c>
       <c r="C94" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D94" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="E94">
         <v>79</v>
@@ -2951,18 +2960,18 @@
         <v>8</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A95" t="s">
-        <v>220</v>
-      </c>
-      <c r="B95" t="s">
-        <v>221</v>
+        <v>127</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>226</v>
       </c>
       <c r="C95" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D95" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="E95">
         <v>53</v>
@@ -2971,18 +2980,18 @@
         <v>7</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A96" t="s">
-        <v>222</v>
-      </c>
-      <c r="B96" t="s">
-        <v>223</v>
+        <v>128</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>227</v>
       </c>
       <c r="C96" t="s">
-        <v>82</v>
+        <v>55</v>
       </c>
       <c r="D96" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E96">
         <v>128</v>
@@ -2991,18 +3000,18 @@
         <v>8</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A97" t="s">
-        <v>224</v>
-      </c>
-      <c r="B97" t="s">
-        <v>225</v>
+        <v>129</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>228</v>
       </c>
       <c r="C97" t="s">
-        <v>209</v>
+        <v>121</v>
       </c>
       <c r="D97" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="E97">
         <v>50</v>
@@ -3011,18 +3020,18 @@
         <v>7</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="98" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A98" t="s">
-        <v>226</v>
-      </c>
-      <c r="B98" t="s">
-        <v>227</v>
+        <v>130</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>229</v>
       </c>
       <c r="C98" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D98" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="E98">
         <v>102</v>
@@ -3031,18 +3040,18 @@
         <v>7</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="99" spans="1:6" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A99" t="s">
-        <v>228</v>
-      </c>
-      <c r="B99" t="s">
-        <v>229</v>
+        <v>131</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>230</v>
       </c>
       <c r="C99" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D99" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="E99">
         <v>71</v>
@@ -3053,16 +3062,16 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A100" t="s">
-        <v>230</v>
-      </c>
-      <c r="B100" t="s">
+        <v>132</v>
+      </c>
+      <c r="B100" s="1" t="s">
         <v>231</v>
       </c>
       <c r="C100" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="D100" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E100">
         <v>149</v>
@@ -3073,16 +3082,16 @@
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A101" t="s">
+        <v>133</v>
+      </c>
+      <c r="B101" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="B101" t="s">
-        <v>233</v>
-      </c>
       <c r="C101" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="D101" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E101">
         <v>89</v>
@@ -3093,5 +3102,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>